<commit_message>
ok for output and baseline comparision
</commit_message>
<xml_diff>
--- a/excel/performance.xlsx
+++ b/excel/performance.xlsx
@@ -37,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -50,6 +50,27 @@
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -425,13 +446,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Orchestrator</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -468,57 +489,240 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Debate</t>
+          <t>No_rag</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.64</v>
+        <v>0.42</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02</v>
+        <v>0.35</v>
       </c>
       <c r="E2" t="n">
-        <v>396.69997</v>
+        <v>0.00377</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>3m39s</t>
+          <t>0m59s</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Rag</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.00728</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1m26s</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n"/>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Rag_keyword</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.00326</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0m45s</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>phi4</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>Debate</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>No_rag</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.00813</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1m38s</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Rag</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.01418</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2m38s</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n"/>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Rag_keyword</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.0185</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>3m17s</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>llama3.3</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Debate</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>No_rag</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.02099</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>4m17s</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n"/>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Rag</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.03613</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>8m7s</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Rag_keyword</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.02204</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>3m36s</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Rag</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>phi4_rag</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>7m41s</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A8:A10"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>